<commit_message>
Update 4. Examen GitHub F. - 3.xlsx
</commit_message>
<xml_diff>
--- a/4. Examen GitHub F. - 3.xlsx
+++ b/4. Examen GitHub F. - 3.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GreenSQA\OneDrive - GreenSQA\Descargas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://greensqa-my.sharepoint.com/personal/mgranda_greensqa_com/Documents/Documentos/GitHub/ProyectoTesting/SegurosGreen/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="68" documentId="8_{02D95A49-5C41-44E4-922A-A692A07D0480}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{1D32C939-CF86-40EB-8242-405F40DB827A}"/>
+  <xr:revisionPtr revIDLastSave="78" documentId="8_{02D95A49-5C41-44E4-922A-A692A07D0480}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A23B6915-DDBD-4879-BA1B-B5774A66B6EF}"/>
   <bookViews>
-    <workbookView xWindow="990" yWindow="0" windowWidth="18210" windowHeight="10920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3705" yWindow="1635" windowWidth="24300" windowHeight="18690" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -203,7 +203,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="73">
   <si>
     <t>*Tiempo medio (En minutos)</t>
   </si>
@@ -407,6 +407,21 @@
   </si>
   <si>
     <t>Hace innecesarias las pruebas automatizadas</t>
+  </si>
+  <si>
+    <t>Git vs GitHub en un proyecto QA</t>
+  </si>
+  <si>
+    <t>Un equipo de QA almacena casos de prueba localmente en sus computadores y desea tener control de cambios y colaboración centralizada. ¿Qué combinación resuelve mejor esta necesidad?</t>
+  </si>
+  <si>
+    <t>Fundamentos GitHub</t>
+  </si>
+  <si>
+    <t>Git para gestionar versiones localmente y GitHub para centralizar y compartir el repositorio.</t>
+  </si>
+  <si>
+    <t>Correcto. Git controla cambios y GitHub facilita colaboración y almacenamiento centralizado.</t>
   </si>
 </sst>
 </file>
@@ -452,7 +467,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -467,15 +482,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -685,24 +695,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AZ988"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="2.6328125" customWidth="1"/>
+    <col min="1" max="1" width="19" customWidth="1"/>
     <col min="2" max="2" width="21" style="1" customWidth="1"/>
     <col min="3" max="3" width="14" style="1" customWidth="1"/>
-    <col min="4" max="4" width="7.81640625" customWidth="1"/>
-    <col min="5" max="5" width="22.6328125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="7.85546875" customWidth="1"/>
+    <col min="5" max="5" width="22.5703125" style="1" customWidth="1"/>
     <col min="6" max="6" width="5" style="1" customWidth="1"/>
     <col min="7" max="7" width="21" style="1" customWidth="1"/>
-    <col min="8" max="8" width="4.90625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="21.36328125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="6.26953125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="19.36328125" style="1" customWidth="1"/>
-    <col min="12" max="12" width="5.54296875" style="1" customWidth="1"/>
-    <col min="13" max="52" width="14.453125" style="1"/>
+    <col min="8" max="8" width="4.85546875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="21.42578125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="6.28515625" style="1" customWidth="1"/>
+    <col min="11" max="11" width="19.42578125" style="1" customWidth="1"/>
+    <col min="12" max="12" width="5.5703125" style="1" customWidth="1"/>
+    <col min="13" max="52" width="14.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -721,7 +731,7 @@
       <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="7" t="s">
         <v>6</v>
       </c>
       <c r="H1" s="3" t="s">
@@ -740,7 +750,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>5</v>
       </c>
@@ -765,7 +775,7 @@
       <c r="L2" s="4"/>
       <c r="M2" s="4"/>
     </row>
-    <row r="3" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>5</v>
       </c>
@@ -775,15 +785,13 @@
       <c r="C3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="6"/>
-      <c r="G3" s="7" t="s">
+      <c r="G3" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="6"/>
-      <c r="I3" s="7" t="s">
+      <c r="I3" s="5" t="s">
         <v>19</v>
       </c>
       <c r="K3" s="5" t="s">
@@ -792,7 +800,7 @@
       <c r="L3" s="4"/>
       <c r="M3" s="4"/>
     </row>
-    <row r="4" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>5</v>
       </c>
@@ -802,22 +810,22 @@
       <c r="C4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="E4" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="F4" s="13"/>
+      <c r="F4" s="10"/>
       <c r="G4" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I4" s="15" t="s">
+      <c r="I4" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="J4" s="14"/>
-      <c r="K4" s="15"/>
+      <c r="J4" s="11"/>
+      <c r="K4" s="12"/>
       <c r="L4" s="4"/>
       <c r="M4" s="4"/>
     </row>
-    <row r="5" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>5</v>
       </c>
@@ -827,23 +835,22 @@
       <c r="C5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="E5" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="G5" s="11" t="s">
+      <c r="G5" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="I5" s="7" t="s">
+      <c r="I5" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="K5" s="6" t="s">
+      <c r="K5" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="L5" s="7"/>
-      <c r="M5" s="6"/>
+      <c r="L5" s="5"/>
       <c r="N5" s="4"/>
     </row>
-    <row r="6" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -859,17 +866,16 @@
       <c r="G6" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="I6" s="7" t="s">
+      <c r="I6" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="K6" s="6" t="s">
+      <c r="K6" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="L6" s="7"/>
-      <c r="M6" s="6"/>
+      <c r="L6" s="5"/>
       <c r="N6" s="4"/>
     </row>
-    <row r="7" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>5</v>
       </c>
@@ -885,16 +891,15 @@
       <c r="G7" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="I7" s="7" t="s">
+      <c r="I7" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="K7" s="6" t="s">
+      <c r="K7" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="L7" s="7"/>
-      <c r="M7" s="6"/>
-    </row>
-    <row r="8" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="L7" s="5"/>
+    </row>
+    <row r="8" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>5</v>
       </c>
@@ -910,16 +915,15 @@
       <c r="G8" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="I8" s="7" t="s">
+      <c r="I8" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="K8" s="6" t="s">
+      <c r="K8" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="L8" s="7"/>
-      <c r="M8" s="6"/>
-    </row>
-    <row r="9" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="L8" s="5"/>
+    </row>
+    <row r="9" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>5</v>
       </c>
@@ -935,16 +939,15 @@
       <c r="G9" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="I9" s="7" t="s">
+      <c r="I9" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="K9" s="6" t="s">
+      <c r="K9" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="L9" s="7"/>
-      <c r="M9" s="6"/>
-    </row>
-    <row r="10" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="L9" s="5"/>
+    </row>
+    <row r="10" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>5</v>
       </c>
@@ -954,23 +957,21 @@
       <c r="C10" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="F10" s="6"/>
       <c r="G10" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="I10" s="7" t="s">
+      <c r="I10" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="K10" s="6" t="s">
+      <c r="K10" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="L10" s="7"/>
-      <c r="M10" s="6"/>
-    </row>
-    <row r="11" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="L10" s="5"/>
+    </row>
+    <row r="11" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>5</v>
       </c>
@@ -980,24 +981,21 @@
       <c r="C11" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="E11" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="F11" s="6"/>
       <c r="G11" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="H11" s="6"/>
-      <c r="I11" s="7" t="s">
+      <c r="I11" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="J11" s="6"/>
-      <c r="K11" s="7" t="s">
+      <c r="K11" s="5" t="s">
         <v>57</v>
       </c>
       <c r="L11" s="4"/>
     </row>
-    <row r="12" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>5</v>
       </c>
@@ -1021,7 +1019,7 @@
       </c>
       <c r="L12" s="4"/>
     </row>
-    <row r="13" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>5</v>
       </c>
@@ -1045,17 +1043,31 @@
       </c>
       <c r="L13" s="4"/>
     </row>
-    <row r="14" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="2"/>
-      <c r="B14" s="4"/>
-      <c r="E14" s="4"/>
+    <row r="14" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="4">
+        <v>2</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>72</v>
+      </c>
       <c r="G14" s="4"/>
       <c r="I14" s="4"/>
       <c r="K14" s="4"/>
       <c r="L14" s="4"/>
     </row>
-    <row r="15" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="2"/>
+    <row r="15" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="4"/>
       <c r="E15" s="4"/>
       <c r="G15" s="4"/>
@@ -1063,7 +1075,7 @@
       <c r="K15" s="4"/>
       <c r="L15" s="4"/>
     </row>
-    <row r="16" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="4"/>
       <c r="E16" s="4"/>
       <c r="G16" s="4"/>
@@ -1071,42 +1083,47 @@
       <c r="K16" s="4"/>
       <c r="L16" s="4"/>
     </row>
-    <row r="17" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F17"/>
       <c r="H17" s="3"/>
       <c r="I17" s="3"/>
     </row>
-    <row r="18" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
       <c r="H18" s="3"/>
     </row>
-    <row r="19" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
     </row>
-    <row r="20" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="4"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
       <c r="H20" s="3"/>
     </row>
-    <row r="21" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="4"/>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
       <c r="H21" s="3"/>
     </row>
-    <row r="22" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="4"/>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
       <c r="H22" s="3"/>
     </row>
-    <row r="23" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="4"/>
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
       <c r="H23" s="3"/>
     </row>
-    <row r="24" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="4"/>
       <c r="B24" s="3"/>
       <c r="D24" s="2"/>
       <c r="E24" s="3"/>
@@ -1114,8 +1131,8 @@
       <c r="G24" s="3"/>
       <c r="H24" s="3"/>
     </row>
-    <row r="25" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="2"/>
+    <row r="25" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="4"/>
       <c r="B25" s="3"/>
       <c r="D25" s="2"/>
       <c r="E25" s="3"/>
@@ -1123,7 +1140,7 @@
       <c r="G25" s="3"/>
       <c r="H25" s="3"/>
     </row>
-    <row r="26" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
       <c r="B26" s="3"/>
       <c r="D26" s="2"/>
@@ -1132,7 +1149,7 @@
       <c r="G26" s="3"/>
       <c r="H26" s="3"/>
     </row>
-    <row r="27" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
       <c r="B27" s="3"/>
       <c r="D27" s="2"/>
@@ -1141,7 +1158,7 @@
       <c r="G27" s="3"/>
       <c r="H27" s="3"/>
     </row>
-    <row r="28" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
       <c r="B28" s="3"/>
       <c r="D28" s="2"/>
@@ -1150,7 +1167,7 @@
       <c r="G28" s="3"/>
       <c r="H28" s="3"/>
     </row>
-    <row r="29" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
       <c r="B29" s="3"/>
       <c r="D29" s="2"/>
@@ -1159,7 +1176,7 @@
       <c r="G29" s="3"/>
       <c r="H29" s="3"/>
     </row>
-    <row r="30" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>
       <c r="B30" s="3"/>
       <c r="D30" s="2"/>
@@ -1168,7 +1185,7 @@
       <c r="G30" s="3"/>
       <c r="H30" s="3"/>
     </row>
-    <row r="31" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2"/>
       <c r="B31" s="3"/>
       <c r="D31" s="2"/>
@@ -1177,7 +1194,7 @@
       <c r="G31" s="3"/>
       <c r="H31" s="3"/>
     </row>
-    <row r="32" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2"/>
       <c r="B32" s="3"/>
       <c r="D32" s="2"/>
@@ -1186,7 +1203,7 @@
       <c r="G32" s="3"/>
       <c r="H32" s="3"/>
     </row>
-    <row r="33" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2"/>
       <c r="B33" s="3"/>
       <c r="D33" s="2"/>
@@ -1195,7 +1212,7 @@
       <c r="G33" s="3"/>
       <c r="H33" s="3"/>
     </row>
-    <row r="34" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2"/>
       <c r="B34" s="3"/>
       <c r="D34" s="2"/>
@@ -1204,7 +1221,7 @@
       <c r="G34" s="3"/>
       <c r="H34" s="3"/>
     </row>
-    <row r="35" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2"/>
       <c r="B35" s="3"/>
       <c r="D35" s="2"/>
@@ -1213,7 +1230,7 @@
       <c r="G35" s="3"/>
       <c r="H35" s="3"/>
     </row>
-    <row r="36" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2"/>
       <c r="B36" s="3"/>
       <c r="D36" s="2"/>
@@ -1222,7 +1239,7 @@
       <c r="G36" s="3"/>
       <c r="H36" s="3"/>
     </row>
-    <row r="37" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2"/>
       <c r="B37" s="3"/>
       <c r="D37" s="2"/>
@@ -1231,7 +1248,7 @@
       <c r="G37" s="3"/>
       <c r="H37" s="3"/>
     </row>
-    <row r="38" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2"/>
       <c r="B38" s="3"/>
       <c r="D38" s="2"/>
@@ -1240,7 +1257,7 @@
       <c r="G38" s="3"/>
       <c r="H38" s="3"/>
     </row>
-    <row r="39" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2"/>
       <c r="B39" s="3"/>
       <c r="D39" s="2"/>
@@ -1249,7 +1266,7 @@
       <c r="G39" s="3"/>
       <c r="H39" s="3"/>
     </row>
-    <row r="40" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2"/>
       <c r="B40" s="3"/>
       <c r="D40" s="2"/>
@@ -1258,7 +1275,7 @@
       <c r="G40" s="3"/>
       <c r="H40" s="3"/>
     </row>
-    <row r="41" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2"/>
       <c r="B41" s="3"/>
       <c r="D41" s="2"/>
@@ -1267,7 +1284,7 @@
       <c r="G41" s="3"/>
       <c r="H41" s="3"/>
     </row>
-    <row r="42" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2"/>
       <c r="B42" s="3"/>
       <c r="D42" s="2"/>
@@ -1276,7 +1293,7 @@
       <c r="G42" s="3"/>
       <c r="H42" s="3"/>
     </row>
-    <row r="43" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2"/>
       <c r="B43" s="3"/>
       <c r="D43" s="2"/>
@@ -1285,7 +1302,7 @@
       <c r="G43" s="3"/>
       <c r="H43" s="3"/>
     </row>
-    <row r="44" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2"/>
       <c r="B44" s="3"/>
       <c r="D44" s="2"/>
@@ -1294,7 +1311,7 @@
       <c r="G44" s="3"/>
       <c r="H44" s="3"/>
     </row>
-    <row r="45" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2"/>
       <c r="B45" s="3"/>
       <c r="D45" s="2"/>
@@ -1303,7 +1320,7 @@
       <c r="G45" s="3"/>
       <c r="H45" s="3"/>
     </row>
-    <row r="46" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2"/>
       <c r="B46" s="3"/>
       <c r="D46" s="2"/>
@@ -1312,7 +1329,7 @@
       <c r="G46" s="3"/>
       <c r="H46" s="3"/>
     </row>
-    <row r="47" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2"/>
       <c r="B47" s="3"/>
       <c r="D47" s="2"/>
@@ -1321,7 +1338,7 @@
       <c r="G47" s="3"/>
       <c r="H47" s="3"/>
     </row>
-    <row r="48" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2"/>
       <c r="B48" s="3"/>
       <c r="D48" s="2"/>
@@ -1330,7 +1347,7 @@
       <c r="G48" s="3"/>
       <c r="H48" s="3"/>
     </row>
-    <row r="49" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2"/>
       <c r="B49" s="3"/>
       <c r="D49" s="2"/>
@@ -1339,7 +1356,7 @@
       <c r="G49" s="3"/>
       <c r="H49" s="3"/>
     </row>
-    <row r="50" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2"/>
       <c r="B50" s="3"/>
       <c r="D50" s="2"/>
@@ -1348,7 +1365,7 @@
       <c r="G50" s="3"/>
       <c r="H50" s="3"/>
     </row>
-    <row r="51" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2"/>
       <c r="B51" s="3"/>
       <c r="D51" s="2"/>
@@ -1357,7 +1374,7 @@
       <c r="G51" s="3"/>
       <c r="H51" s="3"/>
     </row>
-    <row r="52" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2"/>
       <c r="B52" s="3"/>
       <c r="D52" s="2"/>
@@ -1366,7 +1383,7 @@
       <c r="G52" s="3"/>
       <c r="H52" s="3"/>
     </row>
-    <row r="53" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2"/>
       <c r="B53" s="3"/>
       <c r="D53" s="2"/>
@@ -1375,7 +1392,7 @@
       <c r="G53" s="3"/>
       <c r="H53" s="3"/>
     </row>
-    <row r="54" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2"/>
       <c r="B54" s="3"/>
       <c r="D54" s="2"/>
@@ -1384,7 +1401,7 @@
       <c r="G54" s="3"/>
       <c r="H54" s="3"/>
     </row>
-    <row r="55" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2"/>
       <c r="B55" s="3"/>
       <c r="D55" s="2"/>
@@ -1393,7 +1410,7 @@
       <c r="G55" s="3"/>
       <c r="H55" s="3"/>
     </row>
-    <row r="56" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2"/>
       <c r="B56" s="3"/>
       <c r="D56" s="2"/>
@@ -1402,7 +1419,7 @@
       <c r="G56" s="3"/>
       <c r="H56" s="3"/>
     </row>
-    <row r="57" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2"/>
       <c r="B57" s="3"/>
       <c r="D57" s="2"/>
@@ -1411,7 +1428,7 @@
       <c r="G57" s="3"/>
       <c r="H57" s="3"/>
     </row>
-    <row r="58" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2"/>
       <c r="B58" s="3"/>
       <c r="D58" s="2"/>
@@ -1420,7 +1437,7 @@
       <c r="G58" s="3"/>
       <c r="H58" s="3"/>
     </row>
-    <row r="59" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2"/>
       <c r="B59" s="3"/>
       <c r="D59" s="2"/>
@@ -1429,7 +1446,7 @@
       <c r="G59" s="3"/>
       <c r="H59" s="3"/>
     </row>
-    <row r="60" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2"/>
       <c r="B60" s="3"/>
       <c r="D60" s="2"/>
@@ -1438,7 +1455,7 @@
       <c r="G60" s="3"/>
       <c r="H60" s="3"/>
     </row>
-    <row r="61" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2"/>
       <c r="B61" s="3"/>
       <c r="D61" s="2"/>
@@ -1447,7 +1464,7 @@
       <c r="G61" s="3"/>
       <c r="H61" s="3"/>
     </row>
-    <row r="62" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="2"/>
       <c r="B62" s="3"/>
       <c r="D62" s="2"/>
@@ -1456,7 +1473,7 @@
       <c r="G62" s="3"/>
       <c r="H62" s="3"/>
     </row>
-    <row r="63" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="2"/>
       <c r="B63" s="3"/>
       <c r="D63" s="2"/>
@@ -1465,7 +1482,7 @@
       <c r="G63" s="3"/>
       <c r="H63" s="3"/>
     </row>
-    <row r="64" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="2"/>
       <c r="B64" s="3"/>
       <c r="D64" s="2"/>
@@ -1474,7 +1491,7 @@
       <c r="G64" s="3"/>
       <c r="H64" s="3"/>
     </row>
-    <row r="65" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="2"/>
       <c r="B65" s="3"/>
       <c r="D65" s="2"/>
@@ -1483,7 +1500,7 @@
       <c r="G65" s="3"/>
       <c r="H65" s="3"/>
     </row>
-    <row r="66" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2"/>
       <c r="B66" s="3"/>
       <c r="D66" s="2"/>
@@ -1492,7 +1509,7 @@
       <c r="G66" s="3"/>
       <c r="H66" s="3"/>
     </row>
-    <row r="67" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2"/>
       <c r="B67" s="3"/>
       <c r="D67" s="2"/>
@@ -1501,7 +1518,7 @@
       <c r="G67" s="3"/>
       <c r="H67" s="3"/>
     </row>
-    <row r="68" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2"/>
       <c r="B68" s="3"/>
       <c r="D68" s="2"/>
@@ -1510,7 +1527,7 @@
       <c r="G68" s="3"/>
       <c r="H68" s="3"/>
     </row>
-    <row r="69" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="2"/>
       <c r="B69" s="3"/>
       <c r="D69" s="2"/>
@@ -1519,7 +1536,7 @@
       <c r="G69" s="3"/>
       <c r="H69" s="3"/>
     </row>
-    <row r="70" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="2"/>
       <c r="B70" s="3"/>
       <c r="D70" s="2"/>
@@ -1528,7 +1545,7 @@
       <c r="G70" s="3"/>
       <c r="H70" s="3"/>
     </row>
-    <row r="71" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2"/>
       <c r="B71" s="3"/>
       <c r="D71" s="2"/>
@@ -1537,7 +1554,7 @@
       <c r="G71" s="3"/>
       <c r="H71" s="3"/>
     </row>
-    <row r="72" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2"/>
       <c r="B72" s="3"/>
       <c r="D72" s="2"/>
@@ -1546,7 +1563,7 @@
       <c r="G72" s="3"/>
       <c r="H72" s="3"/>
     </row>
-    <row r="73" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="2"/>
       <c r="B73" s="3"/>
       <c r="D73" s="2"/>
@@ -1555,7 +1572,7 @@
       <c r="G73" s="3"/>
       <c r="H73" s="3"/>
     </row>
-    <row r="74" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2"/>
       <c r="B74" s="3"/>
       <c r="D74" s="2"/>
@@ -1564,7 +1581,7 @@
       <c r="G74" s="3"/>
       <c r="H74" s="3"/>
     </row>
-    <row r="75" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="2"/>
       <c r="B75" s="3"/>
       <c r="D75" s="2"/>
@@ -1573,7 +1590,7 @@
       <c r="G75" s="3"/>
       <c r="H75" s="3"/>
     </row>
-    <row r="76" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2"/>
       <c r="B76" s="3"/>
       <c r="D76" s="2"/>
@@ -1582,7 +1599,7 @@
       <c r="G76" s="3"/>
       <c r="H76" s="3"/>
     </row>
-    <row r="77" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="2"/>
       <c r="B77" s="3"/>
       <c r="D77" s="2"/>
@@ -1591,7 +1608,7 @@
       <c r="G77" s="3"/>
       <c r="H77" s="3"/>
     </row>
-    <row r="78" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="2"/>
       <c r="B78" s="3"/>
       <c r="D78" s="2"/>
@@ -1600,7 +1617,7 @@
       <c r="G78" s="3"/>
       <c r="H78" s="3"/>
     </row>
-    <row r="79" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="2"/>
       <c r="B79" s="3"/>
       <c r="D79" s="2"/>
@@ -1609,7 +1626,7 @@
       <c r="G79" s="3"/>
       <c r="H79" s="3"/>
     </row>
-    <row r="80" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2"/>
       <c r="B80" s="3"/>
       <c r="D80" s="2"/>
@@ -1618,7 +1635,7 @@
       <c r="G80" s="3"/>
       <c r="H80" s="3"/>
     </row>
-    <row r="81" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="2"/>
       <c r="B81" s="3"/>
       <c r="D81" s="2"/>
@@ -1627,7 +1644,7 @@
       <c r="G81" s="3"/>
       <c r="H81" s="3"/>
     </row>
-    <row r="82" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="2"/>
       <c r="B82" s="3"/>
       <c r="D82" s="2"/>
@@ -1636,7 +1653,7 @@
       <c r="G82" s="3"/>
       <c r="H82" s="3"/>
     </row>
-    <row r="83" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="2"/>
       <c r="B83" s="3"/>
       <c r="D83" s="2"/>
@@ -1645,7 +1662,7 @@
       <c r="G83" s="3"/>
       <c r="H83" s="3"/>
     </row>
-    <row r="84" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="2"/>
       <c r="B84" s="3"/>
       <c r="D84" s="2"/>
@@ -1654,7 +1671,7 @@
       <c r="G84" s="3"/>
       <c r="H84" s="3"/>
     </row>
-    <row r="85" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="2"/>
       <c r="B85" s="3"/>
       <c r="D85" s="2"/>
@@ -1663,7 +1680,7 @@
       <c r="G85" s="3"/>
       <c r="H85" s="3"/>
     </row>
-    <row r="86" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="2"/>
       <c r="B86" s="3"/>
       <c r="D86" s="2"/>
@@ -1672,7 +1689,7 @@
       <c r="G86" s="3"/>
       <c r="H86" s="3"/>
     </row>
-    <row r="87" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="2"/>
       <c r="B87" s="3"/>
       <c r="D87" s="2"/>
@@ -1681,7 +1698,7 @@
       <c r="G87" s="3"/>
       <c r="H87" s="3"/>
     </row>
-    <row r="88" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="2"/>
       <c r="B88" s="3"/>
       <c r="D88" s="2"/>
@@ -1690,7 +1707,7 @@
       <c r="G88" s="3"/>
       <c r="H88" s="3"/>
     </row>
-    <row r="89" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="2"/>
       <c r="B89" s="3"/>
       <c r="D89" s="2"/>
@@ -1699,7 +1716,7 @@
       <c r="G89" s="3"/>
       <c r="H89" s="3"/>
     </row>
-    <row r="90" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="2"/>
       <c r="B90" s="3"/>
       <c r="D90" s="2"/>
@@ -1708,7 +1725,7 @@
       <c r="G90" s="3"/>
       <c r="H90" s="3"/>
     </row>
-    <row r="91" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="2"/>
       <c r="B91" s="3"/>
       <c r="D91" s="2"/>
@@ -1717,7 +1734,7 @@
       <c r="G91" s="3"/>
       <c r="H91" s="3"/>
     </row>
-    <row r="92" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="2"/>
       <c r="B92" s="3"/>
       <c r="D92" s="2"/>
@@ -1726,7 +1743,7 @@
       <c r="G92" s="3"/>
       <c r="H92" s="3"/>
     </row>
-    <row r="93" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="2"/>
       <c r="B93" s="3"/>
       <c r="D93" s="2"/>
@@ -1735,7 +1752,7 @@
       <c r="G93" s="3"/>
       <c r="H93" s="3"/>
     </row>
-    <row r="94" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="2"/>
       <c r="B94" s="3"/>
       <c r="D94" s="2"/>
@@ -1744,7 +1761,7 @@
       <c r="G94" s="3"/>
       <c r="H94" s="3"/>
     </row>
-    <row r="95" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="2"/>
       <c r="B95" s="3"/>
       <c r="D95" s="2"/>
@@ -1753,7 +1770,7 @@
       <c r="G95" s="3"/>
       <c r="H95" s="3"/>
     </row>
-    <row r="96" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="2"/>
       <c r="B96" s="3"/>
       <c r="D96" s="2"/>
@@ -1762,7 +1779,7 @@
       <c r="G96" s="3"/>
       <c r="H96" s="3"/>
     </row>
-    <row r="97" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="2"/>
       <c r="B97" s="3"/>
       <c r="D97" s="2"/>
@@ -1771,7 +1788,7 @@
       <c r="G97" s="3"/>
       <c r="H97" s="3"/>
     </row>
-    <row r="98" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="2"/>
       <c r="B98" s="3"/>
       <c r="D98" s="2"/>
@@ -1780,7 +1797,7 @@
       <c r="G98" s="3"/>
       <c r="H98" s="3"/>
     </row>
-    <row r="99" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="2"/>
       <c r="B99" s="3"/>
       <c r="D99" s="2"/>
@@ -1789,7 +1806,7 @@
       <c r="G99" s="3"/>
       <c r="H99" s="3"/>
     </row>
-    <row r="100" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="2"/>
       <c r="B100" s="3"/>
       <c r="D100" s="2"/>
@@ -1798,7 +1815,7 @@
       <c r="G100" s="3"/>
       <c r="H100" s="3"/>
     </row>
-    <row r="101" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="2"/>
       <c r="B101" s="3"/>
       <c r="D101" s="2"/>
@@ -1807,7 +1824,7 @@
       <c r="G101" s="3"/>
       <c r="H101" s="3"/>
     </row>
-    <row r="102" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="2"/>
       <c r="B102" s="3"/>
       <c r="D102" s="2"/>
@@ -1816,7 +1833,7 @@
       <c r="G102" s="3"/>
       <c r="H102" s="3"/>
     </row>
-    <row r="103" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="2"/>
       <c r="B103" s="3"/>
       <c r="D103" s="2"/>
@@ -1825,7 +1842,7 @@
       <c r="G103" s="3"/>
       <c r="H103" s="3"/>
     </row>
-    <row r="104" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="2"/>
       <c r="B104" s="3"/>
       <c r="D104" s="2"/>
@@ -1834,7 +1851,7 @@
       <c r="G104" s="3"/>
       <c r="H104" s="3"/>
     </row>
-    <row r="105" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="2"/>
       <c r="B105" s="3"/>
       <c r="D105" s="2"/>
@@ -1843,7 +1860,7 @@
       <c r="G105" s="3"/>
       <c r="H105" s="3"/>
     </row>
-    <row r="106" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="2"/>
       <c r="B106" s="3"/>
       <c r="D106" s="2"/>
@@ -1852,7 +1869,7 @@
       <c r="G106" s="3"/>
       <c r="H106" s="3"/>
     </row>
-    <row r="107" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="2"/>
       <c r="B107" s="3"/>
       <c r="D107" s="2"/>
@@ -1861,7 +1878,7 @@
       <c r="G107" s="3"/>
       <c r="H107" s="3"/>
     </row>
-    <row r="108" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="2"/>
       <c r="B108" s="3"/>
       <c r="D108" s="2"/>
@@ -1870,7 +1887,7 @@
       <c r="G108" s="3"/>
       <c r="H108" s="3"/>
     </row>
-    <row r="109" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="2"/>
       <c r="B109" s="3"/>
       <c r="D109" s="2"/>
@@ -1879,7 +1896,7 @@
       <c r="G109" s="3"/>
       <c r="H109" s="3"/>
     </row>
-    <row r="110" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="2"/>
       <c r="B110" s="3"/>
       <c r="D110" s="2"/>
@@ -1888,7 +1905,7 @@
       <c r="G110" s="3"/>
       <c r="H110" s="3"/>
     </row>
-    <row r="111" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="2"/>
       <c r="B111" s="3"/>
       <c r="D111" s="2"/>
@@ -1897,7 +1914,7 @@
       <c r="G111" s="3"/>
       <c r="H111" s="3"/>
     </row>
-    <row r="112" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="2"/>
       <c r="B112" s="3"/>
       <c r="D112" s="2"/>
@@ -1906,7 +1923,7 @@
       <c r="G112" s="3"/>
       <c r="H112" s="3"/>
     </row>
-    <row r="113" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="2"/>
       <c r="B113" s="3"/>
       <c r="D113" s="2"/>
@@ -1915,7 +1932,7 @@
       <c r="G113" s="3"/>
       <c r="H113" s="3"/>
     </row>
-    <row r="114" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114" s="2"/>
       <c r="B114" s="3"/>
       <c r="D114" s="2"/>
@@ -1924,7 +1941,7 @@
       <c r="G114" s="3"/>
       <c r="H114" s="3"/>
     </row>
-    <row r="115" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="2"/>
       <c r="B115" s="3"/>
       <c r="D115" s="2"/>
@@ -1933,7 +1950,7 @@
       <c r="G115" s="3"/>
       <c r="H115" s="3"/>
     </row>
-    <row r="116" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="2"/>
       <c r="B116" s="3"/>
       <c r="D116" s="2"/>
@@ -1942,7 +1959,7 @@
       <c r="G116" s="3"/>
       <c r="H116" s="3"/>
     </row>
-    <row r="117" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="2"/>
       <c r="B117" s="3"/>
       <c r="D117" s="2"/>
@@ -1951,7 +1968,7 @@
       <c r="G117" s="3"/>
       <c r="H117" s="3"/>
     </row>
-    <row r="118" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118" s="2"/>
       <c r="B118" s="3"/>
       <c r="D118" s="2"/>
@@ -1960,7 +1977,7 @@
       <c r="G118" s="3"/>
       <c r="H118" s="3"/>
     </row>
-    <row r="119" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="2"/>
       <c r="B119" s="3"/>
       <c r="D119" s="2"/>
@@ -1969,7 +1986,7 @@
       <c r="G119" s="3"/>
       <c r="H119" s="3"/>
     </row>
-    <row r="120" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="2"/>
       <c r="B120" s="3"/>
       <c r="D120" s="2"/>
@@ -1978,7 +1995,7 @@
       <c r="G120" s="3"/>
       <c r="H120" s="3"/>
     </row>
-    <row r="121" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="2"/>
       <c r="B121" s="3"/>
       <c r="D121" s="2"/>
@@ -1987,7 +2004,7 @@
       <c r="G121" s="3"/>
       <c r="H121" s="3"/>
     </row>
-    <row r="122" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="2"/>
       <c r="B122" s="3"/>
       <c r="D122" s="2"/>
@@ -1996,7 +2013,7 @@
       <c r="G122" s="3"/>
       <c r="H122" s="3"/>
     </row>
-    <row r="123" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123" s="2"/>
       <c r="B123" s="3"/>
       <c r="D123" s="2"/>
@@ -2005,7 +2022,7 @@
       <c r="G123" s="3"/>
       <c r="H123" s="3"/>
     </row>
-    <row r="124" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124" s="2"/>
       <c r="B124" s="3"/>
       <c r="D124" s="2"/>
@@ -2014,7 +2031,7 @@
       <c r="G124" s="3"/>
       <c r="H124" s="3"/>
     </row>
-    <row r="125" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="2"/>
       <c r="B125" s="3"/>
       <c r="D125" s="2"/>
@@ -2023,7 +2040,7 @@
       <c r="G125" s="3"/>
       <c r="H125" s="3"/>
     </row>
-    <row r="126" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126" s="2"/>
       <c r="B126" s="3"/>
       <c r="D126" s="2"/>
@@ -2032,7 +2049,7 @@
       <c r="G126" s="3"/>
       <c r="H126" s="3"/>
     </row>
-    <row r="127" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127" s="2"/>
       <c r="B127" s="3"/>
       <c r="D127" s="2"/>
@@ -2041,7 +2058,7 @@
       <c r="G127" s="3"/>
       <c r="H127" s="3"/>
     </row>
-    <row r="128" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128" s="2"/>
       <c r="B128" s="3"/>
       <c r="D128" s="2"/>
@@ -2050,7 +2067,7 @@
       <c r="G128" s="3"/>
       <c r="H128" s="3"/>
     </row>
-    <row r="129" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="2"/>
       <c r="B129" s="3"/>
       <c r="D129" s="2"/>
@@ -2059,7 +2076,7 @@
       <c r="G129" s="3"/>
       <c r="H129" s="3"/>
     </row>
-    <row r="130" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="2"/>
       <c r="B130" s="3"/>
       <c r="D130" s="2"/>
@@ -2068,7 +2085,7 @@
       <c r="G130" s="3"/>
       <c r="H130" s="3"/>
     </row>
-    <row r="131" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="2"/>
       <c r="B131" s="3"/>
       <c r="D131" s="2"/>
@@ -2077,7 +2094,7 @@
       <c r="G131" s="3"/>
       <c r="H131" s="3"/>
     </row>
-    <row r="132" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="2"/>
       <c r="B132" s="3"/>
       <c r="D132" s="2"/>
@@ -2086,7 +2103,7 @@
       <c r="G132" s="3"/>
       <c r="H132" s="3"/>
     </row>
-    <row r="133" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" s="2"/>
       <c r="B133" s="3"/>
       <c r="D133" s="2"/>
@@ -2095,7 +2112,7 @@
       <c r="G133" s="3"/>
       <c r="H133" s="3"/>
     </row>
-    <row r="134" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A134" s="2"/>
       <c r="B134" s="3"/>
       <c r="D134" s="2"/>
@@ -2104,7 +2121,7 @@
       <c r="G134" s="3"/>
       <c r="H134" s="3"/>
     </row>
-    <row r="135" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A135" s="2"/>
       <c r="B135" s="3"/>
       <c r="D135" s="2"/>
@@ -2113,7 +2130,7 @@
       <c r="G135" s="3"/>
       <c r="H135" s="3"/>
     </row>
-    <row r="136" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A136" s="2"/>
       <c r="B136" s="3"/>
       <c r="D136" s="2"/>
@@ -2122,7 +2139,7 @@
       <c r="G136" s="3"/>
       <c r="H136" s="3"/>
     </row>
-    <row r="137" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137" s="2"/>
       <c r="B137" s="3"/>
       <c r="D137" s="2"/>
@@ -2131,7 +2148,7 @@
       <c r="G137" s="3"/>
       <c r="H137" s="3"/>
     </row>
-    <row r="138" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A138" s="2"/>
       <c r="B138" s="3"/>
       <c r="D138" s="2"/>
@@ -2140,7 +2157,7 @@
       <c r="G138" s="3"/>
       <c r="H138" s="3"/>
     </row>
-    <row r="139" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139" s="2"/>
       <c r="B139" s="3"/>
       <c r="D139" s="2"/>
@@ -2149,7 +2166,7 @@
       <c r="G139" s="3"/>
       <c r="H139" s="3"/>
     </row>
-    <row r="140" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140" s="2"/>
       <c r="B140" s="3"/>
       <c r="D140" s="2"/>
@@ -2158,7 +2175,7 @@
       <c r="G140" s="3"/>
       <c r="H140" s="3"/>
     </row>
-    <row r="141" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A141" s="2"/>
       <c r="B141" s="3"/>
       <c r="D141" s="2"/>
@@ -2167,7 +2184,7 @@
       <c r="G141" s="3"/>
       <c r="H141" s="3"/>
     </row>
-    <row r="142" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A142" s="2"/>
       <c r="B142" s="3"/>
       <c r="D142" s="2"/>
@@ -2176,7 +2193,7 @@
       <c r="G142" s="3"/>
       <c r="H142" s="3"/>
     </row>
-    <row r="143" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143" s="2"/>
       <c r="B143" s="3"/>
       <c r="D143" s="2"/>
@@ -2185,7 +2202,7 @@
       <c r="G143" s="3"/>
       <c r="H143" s="3"/>
     </row>
-    <row r="144" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A144" s="2"/>
       <c r="B144" s="3"/>
       <c r="D144" s="2"/>
@@ -2194,7 +2211,7 @@
       <c r="G144" s="3"/>
       <c r="H144" s="3"/>
     </row>
-    <row r="145" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A145" s="2"/>
       <c r="B145" s="3"/>
       <c r="D145" s="2"/>
@@ -2203,7 +2220,7 @@
       <c r="G145" s="3"/>
       <c r="H145" s="3"/>
     </row>
-    <row r="146" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A146" s="2"/>
       <c r="B146" s="3"/>
       <c r="D146" s="2"/>
@@ -2212,7 +2229,7 @@
       <c r="G146" s="3"/>
       <c r="H146" s="3"/>
     </row>
-    <row r="147" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A147" s="2"/>
       <c r="B147" s="3"/>
       <c r="D147" s="2"/>
@@ -2221,7 +2238,7 @@
       <c r="G147" s="3"/>
       <c r="H147" s="3"/>
     </row>
-    <row r="148" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A148" s="2"/>
       <c r="B148" s="3"/>
       <c r="D148" s="2"/>
@@ -2230,7 +2247,7 @@
       <c r="G148" s="3"/>
       <c r="H148" s="3"/>
     </row>
-    <row r="149" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A149" s="2"/>
       <c r="B149" s="3"/>
       <c r="D149" s="2"/>
@@ -2239,7 +2256,7 @@
       <c r="G149" s="3"/>
       <c r="H149" s="3"/>
     </row>
-    <row r="150" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A150" s="2"/>
       <c r="B150" s="3"/>
       <c r="D150" s="2"/>
@@ -2248,7 +2265,7 @@
       <c r="G150" s="3"/>
       <c r="H150" s="3"/>
     </row>
-    <row r="151" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A151" s="2"/>
       <c r="B151" s="3"/>
       <c r="D151" s="2"/>
@@ -2257,7 +2274,7 @@
       <c r="G151" s="3"/>
       <c r="H151" s="3"/>
     </row>
-    <row r="152" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A152" s="2"/>
       <c r="B152" s="3"/>
       <c r="D152" s="2"/>
@@ -2266,7 +2283,7 @@
       <c r="G152" s="3"/>
       <c r="H152" s="3"/>
     </row>
-    <row r="153" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="2"/>
       <c r="B153" s="3"/>
       <c r="D153" s="2"/>
@@ -2275,7 +2292,7 @@
       <c r="G153" s="3"/>
       <c r="H153" s="3"/>
     </row>
-    <row r="154" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A154" s="2"/>
       <c r="B154" s="3"/>
       <c r="D154" s="2"/>
@@ -2284,7 +2301,7 @@
       <c r="G154" s="3"/>
       <c r="H154" s="3"/>
     </row>
-    <row r="155" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A155" s="2"/>
       <c r="B155" s="3"/>
       <c r="D155" s="2"/>
@@ -2293,7 +2310,7 @@
       <c r="G155" s="3"/>
       <c r="H155" s="3"/>
     </row>
-    <row r="156" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A156" s="2"/>
       <c r="B156" s="3"/>
       <c r="D156" s="2"/>
@@ -2302,7 +2319,7 @@
       <c r="G156" s="3"/>
       <c r="H156" s="3"/>
     </row>
-    <row r="157" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A157" s="2"/>
       <c r="B157" s="3"/>
       <c r="D157" s="2"/>
@@ -2311,7 +2328,7 @@
       <c r="G157" s="3"/>
       <c r="H157" s="3"/>
     </row>
-    <row r="158" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A158" s="2"/>
       <c r="B158" s="3"/>
       <c r="D158" s="2"/>
@@ -2320,7 +2337,7 @@
       <c r="G158" s="3"/>
       <c r="H158" s="3"/>
     </row>
-    <row r="159" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A159" s="2"/>
       <c r="B159" s="3"/>
       <c r="D159" s="2"/>
@@ -2329,7 +2346,7 @@
       <c r="G159" s="3"/>
       <c r="H159" s="3"/>
     </row>
-    <row r="160" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A160" s="2"/>
       <c r="B160" s="3"/>
       <c r="D160" s="2"/>
@@ -2338,7 +2355,7 @@
       <c r="G160" s="3"/>
       <c r="H160" s="3"/>
     </row>
-    <row r="161" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A161" s="2"/>
       <c r="B161" s="3"/>
       <c r="D161" s="2"/>
@@ -2347,7 +2364,7 @@
       <c r="G161" s="3"/>
       <c r="H161" s="3"/>
     </row>
-    <row r="162" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A162" s="2"/>
       <c r="B162" s="3"/>
       <c r="D162" s="2"/>
@@ -2356,7 +2373,7 @@
       <c r="G162" s="3"/>
       <c r="H162" s="3"/>
     </row>
-    <row r="163" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A163" s="2"/>
       <c r="B163" s="3"/>
       <c r="D163" s="2"/>
@@ -2365,7 +2382,7 @@
       <c r="G163" s="3"/>
       <c r="H163" s="3"/>
     </row>
-    <row r="164" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A164" s="2"/>
       <c r="B164" s="3"/>
       <c r="D164" s="2"/>
@@ -2374,7 +2391,7 @@
       <c r="G164" s="3"/>
       <c r="H164" s="3"/>
     </row>
-    <row r="165" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A165" s="2"/>
       <c r="B165" s="3"/>
       <c r="D165" s="2"/>
@@ -2383,7 +2400,7 @@
       <c r="G165" s="3"/>
       <c r="H165" s="3"/>
     </row>
-    <row r="166" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A166" s="2"/>
       <c r="B166" s="3"/>
       <c r="D166" s="2"/>
@@ -2392,7 +2409,7 @@
       <c r="G166" s="3"/>
       <c r="H166" s="3"/>
     </row>
-    <row r="167" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A167" s="2"/>
       <c r="B167" s="3"/>
       <c r="D167" s="2"/>
@@ -2401,7 +2418,7 @@
       <c r="G167" s="3"/>
       <c r="H167" s="3"/>
     </row>
-    <row r="168" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A168" s="2"/>
       <c r="B168" s="3"/>
       <c r="D168" s="2"/>
@@ -2410,7 +2427,7 @@
       <c r="G168" s="3"/>
       <c r="H168" s="3"/>
     </row>
-    <row r="169" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A169" s="2"/>
       <c r="B169" s="3"/>
       <c r="D169" s="2"/>
@@ -2419,7 +2436,7 @@
       <c r="G169" s="3"/>
       <c r="H169" s="3"/>
     </row>
-    <row r="170" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A170" s="2"/>
       <c r="B170" s="3"/>
       <c r="D170" s="2"/>
@@ -2428,7 +2445,7 @@
       <c r="G170" s="3"/>
       <c r="H170" s="3"/>
     </row>
-    <row r="171" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A171" s="2"/>
       <c r="B171" s="3"/>
       <c r="D171" s="2"/>
@@ -2437,7 +2454,7 @@
       <c r="G171" s="3"/>
       <c r="H171" s="3"/>
     </row>
-    <row r="172" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A172" s="2"/>
       <c r="B172" s="3"/>
       <c r="D172" s="2"/>
@@ -2446,7 +2463,7 @@
       <c r="G172" s="3"/>
       <c r="H172" s="3"/>
     </row>
-    <row r="173" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A173" s="2"/>
       <c r="B173" s="3"/>
       <c r="D173" s="2"/>
@@ -2455,7 +2472,7 @@
       <c r="G173" s="3"/>
       <c r="H173" s="3"/>
     </row>
-    <row r="174" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A174" s="2"/>
       <c r="B174" s="3"/>
       <c r="D174" s="2"/>
@@ -2464,7 +2481,7 @@
       <c r="G174" s="3"/>
       <c r="H174" s="3"/>
     </row>
-    <row r="175" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A175" s="2"/>
       <c r="B175" s="3"/>
       <c r="D175" s="2"/>
@@ -2473,7 +2490,7 @@
       <c r="G175" s="3"/>
       <c r="H175" s="3"/>
     </row>
-    <row r="176" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A176" s="2"/>
       <c r="B176" s="3"/>
       <c r="D176" s="2"/>
@@ -2482,7 +2499,7 @@
       <c r="G176" s="3"/>
       <c r="H176" s="3"/>
     </row>
-    <row r="177" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A177" s="2"/>
       <c r="B177" s="3"/>
       <c r="D177" s="2"/>
@@ -2491,7 +2508,7 @@
       <c r="G177" s="3"/>
       <c r="H177" s="3"/>
     </row>
-    <row r="178" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A178" s="2"/>
       <c r="B178" s="3"/>
       <c r="D178" s="2"/>
@@ -2500,7 +2517,7 @@
       <c r="G178" s="3"/>
       <c r="H178" s="3"/>
     </row>
-    <row r="179" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A179" s="2"/>
       <c r="B179" s="3"/>
       <c r="D179" s="2"/>
@@ -2509,7 +2526,7 @@
       <c r="G179" s="3"/>
       <c r="H179" s="3"/>
     </row>
-    <row r="180" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A180" s="2"/>
       <c r="B180" s="3"/>
       <c r="D180" s="2"/>
@@ -2518,7 +2535,7 @@
       <c r="G180" s="3"/>
       <c r="H180" s="3"/>
     </row>
-    <row r="181" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A181" s="2"/>
       <c r="B181" s="3"/>
       <c r="D181" s="2"/>
@@ -2527,7 +2544,7 @@
       <c r="G181" s="3"/>
       <c r="H181" s="3"/>
     </row>
-    <row r="182" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A182" s="2"/>
       <c r="B182" s="3"/>
       <c r="D182" s="2"/>
@@ -2536,7 +2553,7 @@
       <c r="G182" s="3"/>
       <c r="H182" s="3"/>
     </row>
-    <row r="183" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A183" s="2"/>
       <c r="B183" s="3"/>
       <c r="D183" s="2"/>
@@ -2545,7 +2562,7 @@
       <c r="G183" s="3"/>
       <c r="H183" s="3"/>
     </row>
-    <row r="184" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A184" s="2"/>
       <c r="B184" s="3"/>
       <c r="D184" s="2"/>
@@ -2554,7 +2571,7 @@
       <c r="G184" s="3"/>
       <c r="H184" s="3"/>
     </row>
-    <row r="185" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A185" s="2"/>
       <c r="B185" s="3"/>
       <c r="D185" s="2"/>
@@ -2563,7 +2580,7 @@
       <c r="G185" s="3"/>
       <c r="H185" s="3"/>
     </row>
-    <row r="186" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A186" s="2"/>
       <c r="B186" s="3"/>
       <c r="D186" s="2"/>
@@ -2572,7 +2589,7 @@
       <c r="G186" s="3"/>
       <c r="H186" s="3"/>
     </row>
-    <row r="187" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A187" s="2"/>
       <c r="B187" s="3"/>
       <c r="D187" s="2"/>
@@ -2581,7 +2598,7 @@
       <c r="G187" s="3"/>
       <c r="H187" s="3"/>
     </row>
-    <row r="188" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A188" s="2"/>
       <c r="B188" s="3"/>
       <c r="D188" s="2"/>
@@ -2590,7 +2607,7 @@
       <c r="G188" s="3"/>
       <c r="H188" s="3"/>
     </row>
-    <row r="189" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A189" s="2"/>
       <c r="B189" s="3"/>
       <c r="D189" s="2"/>
@@ -2599,7 +2616,7 @@
       <c r="G189" s="3"/>
       <c r="H189" s="3"/>
     </row>
-    <row r="190" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A190" s="2"/>
       <c r="B190" s="3"/>
       <c r="D190" s="2"/>
@@ -2608,7 +2625,7 @@
       <c r="G190" s="3"/>
       <c r="H190" s="3"/>
     </row>
-    <row r="191" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A191" s="2"/>
       <c r="B191" s="3"/>
       <c r="D191" s="2"/>
@@ -2617,7 +2634,7 @@
       <c r="G191" s="3"/>
       <c r="H191" s="3"/>
     </row>
-    <row r="192" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A192" s="2"/>
       <c r="B192" s="3"/>
       <c r="D192" s="2"/>
@@ -2626,7 +2643,7 @@
       <c r="G192" s="3"/>
       <c r="H192" s="3"/>
     </row>
-    <row r="193" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A193" s="2"/>
       <c r="B193" s="3"/>
       <c r="D193" s="2"/>
@@ -2635,7 +2652,7 @@
       <c r="G193" s="3"/>
       <c r="H193" s="3"/>
     </row>
-    <row r="194" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A194" s="2"/>
       <c r="B194" s="3"/>
       <c r="D194" s="2"/>
@@ -2644,7 +2661,7 @@
       <c r="G194" s="3"/>
       <c r="H194" s="3"/>
     </row>
-    <row r="195" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A195" s="2"/>
       <c r="B195" s="3"/>
       <c r="D195" s="2"/>
@@ -2653,7 +2670,7 @@
       <c r="G195" s="3"/>
       <c r="H195" s="3"/>
     </row>
-    <row r="196" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A196" s="2"/>
       <c r="B196" s="3"/>
       <c r="D196" s="2"/>
@@ -2662,7 +2679,7 @@
       <c r="G196" s="3"/>
       <c r="H196" s="3"/>
     </row>
-    <row r="197" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A197" s="2"/>
       <c r="B197" s="3"/>
       <c r="D197" s="2"/>
@@ -2671,7 +2688,7 @@
       <c r="G197" s="3"/>
       <c r="H197" s="3"/>
     </row>
-    <row r="198" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A198" s="2"/>
       <c r="B198" s="3"/>
       <c r="D198" s="2"/>
@@ -2680,7 +2697,7 @@
       <c r="G198" s="3"/>
       <c r="H198" s="3"/>
     </row>
-    <row r="199" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A199" s="2"/>
       <c r="B199" s="3"/>
       <c r="D199" s="2"/>
@@ -2689,7 +2706,7 @@
       <c r="G199" s="3"/>
       <c r="H199" s="3"/>
     </row>
-    <row r="200" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A200" s="2"/>
       <c r="B200" s="3"/>
       <c r="D200" s="2"/>
@@ -2698,7 +2715,7 @@
       <c r="G200" s="3"/>
       <c r="H200" s="3"/>
     </row>
-    <row r="201" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A201" s="2"/>
       <c r="B201" s="3"/>
       <c r="D201" s="2"/>
@@ -2707,7 +2724,7 @@
       <c r="G201" s="3"/>
       <c r="H201" s="3"/>
     </row>
-    <row r="202" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A202" s="2"/>
       <c r="B202" s="3"/>
       <c r="D202" s="2"/>
@@ -2716,7 +2733,7 @@
       <c r="G202" s="3"/>
       <c r="H202" s="3"/>
     </row>
-    <row r="203" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A203" s="2"/>
       <c r="B203" s="3"/>
       <c r="D203" s="2"/>
@@ -2725,7 +2742,7 @@
       <c r="G203" s="3"/>
       <c r="H203" s="3"/>
     </row>
-    <row r="204" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A204" s="2"/>
       <c r="B204" s="3"/>
       <c r="D204" s="2"/>
@@ -2734,7 +2751,7 @@
       <c r="G204" s="3"/>
       <c r="H204" s="3"/>
     </row>
-    <row r="205" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A205" s="2"/>
       <c r="B205" s="3"/>
       <c r="D205" s="2"/>
@@ -2743,7 +2760,7 @@
       <c r="G205" s="3"/>
       <c r="H205" s="3"/>
     </row>
-    <row r="206" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A206" s="2"/>
       <c r="B206" s="3"/>
       <c r="D206" s="2"/>
@@ -2752,7 +2769,7 @@
       <c r="G206" s="3"/>
       <c r="H206" s="3"/>
     </row>
-    <row r="207" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A207" s="2"/>
       <c r="B207" s="3"/>
       <c r="D207" s="2"/>
@@ -2761,790 +2778,790 @@
       <c r="G207" s="3"/>
       <c r="H207" s="3"/>
     </row>
-    <row r="208" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A208" s="2"/>
       <c r="H208" s="3"/>
     </row>
-    <row r="209" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="210" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="211" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="212" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="213" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="214" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="215" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="216" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="217" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="218" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="219" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="220" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="221" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="222" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="223" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="224" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="225" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="226" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="227" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="228" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="229" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="230" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="231" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="232" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="233" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="234" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="235" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="236" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="237" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="238" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="239" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="240" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="241" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="242" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="243" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="244" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="245" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="246" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="247" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="248" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="249" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="250" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="251" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="252" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="253" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="254" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="255" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="256" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="257" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="258" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="259" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="260" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="261" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="262" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="263" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="264" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="265" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="266" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="267" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="268" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="269" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="270" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="271" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="272" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="273" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="274" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="275" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="276" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="277" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="278" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="279" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="280" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="281" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="282" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="283" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="284" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="285" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="286" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="287" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="288" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="289" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="290" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="291" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="292" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="293" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="294" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="295" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="296" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="297" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="298" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="299" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="300" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="301" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="302" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="303" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="304" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="305" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="306" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="307" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="308" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="309" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="310" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="311" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="312" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="313" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="314" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="315" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="316" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="317" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="318" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="319" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="320" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="321" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="322" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="323" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="324" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="325" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="326" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="327" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="328" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="329" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="330" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="331" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="332" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="333" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="334" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="335" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="336" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="337" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="338" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="339" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="340" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="341" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="342" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="343" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="344" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="345" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="346" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="347" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="348" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="349" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="350" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="351" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="352" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="353" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="354" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="355" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="356" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="357" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="358" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="359" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="360" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="361" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="362" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="363" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="364" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="365" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="366" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="367" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="368" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="369" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="370" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="371" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="372" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="373" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="374" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="375" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="376" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="377" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="378" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="379" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="380" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="381" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="382" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="383" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="384" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="385" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="386" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="387" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="388" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="389" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="390" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="391" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="392" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="393" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="394" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="395" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="396" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="397" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="398" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="399" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="400" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="401" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="402" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="403" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="404" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="405" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="406" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="407" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="408" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="409" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="410" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="411" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="412" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="413" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="414" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="415" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="416" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="417" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="418" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="419" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="420" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="421" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="422" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="423" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="424" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="425" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="426" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="427" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="428" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="429" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="430" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="431" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="432" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="433" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="434" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="435" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="436" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="437" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="438" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="439" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="440" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="441" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="442" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="443" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="444" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="445" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="446" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="447" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="448" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="449" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="450" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="451" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="452" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="453" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="454" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="455" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="456" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="457" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="458" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="459" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="460" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="461" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="462" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="463" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="464" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="465" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="466" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="467" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="468" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="469" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="470" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="471" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="472" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="473" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="474" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="475" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="476" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="477" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="478" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="479" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="480" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="481" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="482" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="483" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="484" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="485" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="486" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="487" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="488" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="489" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="490" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="491" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="492" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="493" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="494" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="495" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="496" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="497" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="498" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="499" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="500" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="501" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="502" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="503" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="504" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="505" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="506" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="507" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="508" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="509" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="510" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="511" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="512" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="513" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="514" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="515" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="516" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="517" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="518" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="519" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="520" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="521" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="522" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="523" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="524" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="525" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="526" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="527" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="528" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="529" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="530" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="531" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="532" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="533" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="534" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="535" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="536" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="537" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="538" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="539" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="540" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="541" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="542" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="543" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="544" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="545" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="546" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="547" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="548" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="549" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="550" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="551" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="552" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="553" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="554" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="555" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="556" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="557" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="558" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="559" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="560" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="561" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="562" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="563" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="564" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="565" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="566" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="567" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="568" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="569" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="570" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="571" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="572" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="573" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="574" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="575" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="576" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="577" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="578" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="579" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="580" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="581" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="582" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="583" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="584" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="585" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="586" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="587" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="588" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="589" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="590" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="591" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="592" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="593" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="594" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="595" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="596" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="597" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="598" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="599" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="600" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="601" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="602" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="603" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="604" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="605" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="606" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="607" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="608" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="609" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="610" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="611" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="612" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="613" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="614" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="615" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="616" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="617" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="618" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="619" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="620" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="621" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="622" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="623" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="624" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="625" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="626" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="627" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="628" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="629" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="630" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="631" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="632" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="633" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="634" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="635" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="636" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="637" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="638" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="639" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="640" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="641" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="642" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="643" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="644" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="645" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="646" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="647" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="648" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="649" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="650" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="651" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="652" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="653" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="654" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="655" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="656" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="657" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="658" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="659" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="660" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="661" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="662" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="663" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="664" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="665" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="666" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="667" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="668" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="669" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="670" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="671" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="672" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="673" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="674" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="675" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="676" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="677" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="678" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="679" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="680" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="681" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="682" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="683" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="684" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="685" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="686" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="687" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="688" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="689" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="690" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="691" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="692" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="693" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="694" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="695" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="696" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="697" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="698" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="699" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="700" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="701" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="702" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="703" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="704" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="705" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="706" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="707" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="708" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="709" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="710" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="711" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="712" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="713" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="714" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="715" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="716" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="717" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="718" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="719" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="720" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="721" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="722" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="723" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="724" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="725" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="726" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="727" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="728" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="729" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="730" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="731" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="732" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="733" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="734" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="735" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="736" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="737" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="738" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="739" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="740" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="741" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="742" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="743" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="744" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="745" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="746" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="747" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="748" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="749" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="750" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="751" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="752" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="753" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="754" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="755" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="756" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="757" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="758" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="759" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="760" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="761" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="762" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="763" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="764" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="765" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="766" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="767" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="768" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="769" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="770" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="771" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="772" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="773" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="774" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="775" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="776" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="777" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="778" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="779" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="780" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="781" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="782" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="783" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="784" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="785" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="786" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="787" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="788" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="789" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="790" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="791" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="792" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="793" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="794" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="795" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="796" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="797" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="798" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="799" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="800" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="801" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="802" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="803" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="804" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="805" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="806" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="807" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="808" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="809" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="810" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="811" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="812" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="813" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="814" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="815" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="816" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="817" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="818" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="819" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="820" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="821" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="822" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="823" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="824" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="825" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="826" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="827" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="828" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="829" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="830" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="831" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="832" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="833" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="834" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="835" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="836" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="837" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="838" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="839" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="840" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="841" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="842" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="843" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="844" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="845" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="846" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="847" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="848" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="849" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="850" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="851" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="852" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="853" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="854" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="855" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="856" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="857" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="858" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="859" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="860" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="861" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="862" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="863" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="864" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="865" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="866" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="867" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="868" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="869" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="870" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="871" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="872" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="873" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="874" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="875" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="876" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="877" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="878" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="879" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="880" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="881" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="882" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="883" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="884" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="885" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="886" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="887" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="888" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="889" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="890" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="891" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="892" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="893" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="894" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="895" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="896" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="897" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="898" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="899" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="900" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="901" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="902" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="903" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="904" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="905" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="906" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="907" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="908" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="909" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="910" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="911" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="912" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="913" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="914" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="915" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="916" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="917" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="918" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="919" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="920" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="921" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="922" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="923" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="924" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="925" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="926" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="927" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="928" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="929" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="930" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="931" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="932" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="933" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="934" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="935" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="936" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="937" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="938" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="939" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="940" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="941" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="942" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="943" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="944" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="945" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="946" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="947" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="948" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="949" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="950" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="951" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="952" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="953" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="954" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="955" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="956" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="957" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="958" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="959" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="960" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="961" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="962" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="963" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="964" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="965" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="966" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="967" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="968" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="969" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="970" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="971" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="972" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="973" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="974" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="975" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="976" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="977" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="978" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="979" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="980" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="981" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="982" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="983" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="984" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="985" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="986" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="987" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="988" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="209" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="210" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="211" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="212" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="213" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="214" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="215" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="216" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="217" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="218" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="219" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="220" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="221" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="222" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="223" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="224" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="225" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="226" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="227" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="228" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="229" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="230" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="231" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="232" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="233" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="234" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="235" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="236" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="237" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="238" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="239" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="240" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="241" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="242" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="243" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="244" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="245" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="246" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="247" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="248" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="249" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="250" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="251" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="252" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="253" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="254" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="255" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="256" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="257" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="258" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="259" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="260" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="261" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="262" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="263" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="264" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="265" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="266" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="267" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="268" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="269" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="270" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="271" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="272" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="273" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="274" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="275" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="276" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="277" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="278" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="279" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="280" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="281" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="282" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="283" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="284" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="285" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="286" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="287" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="288" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="289" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="290" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="291" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="292" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="293" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="294" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="295" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="296" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="297" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="298" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="299" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="300" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="301" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="302" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="303" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="304" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="305" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="306" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="307" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="308" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="309" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="310" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="311" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="312" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="313" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="314" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="315" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="316" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="317" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="318" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="319" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="320" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="321" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="322" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="323" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="324" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="325" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="326" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="327" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="328" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="329" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="330" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="331" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="332" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="333" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="334" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="335" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="336" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="337" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="338" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="339" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="340" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="341" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="342" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="343" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="344" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="345" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="346" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="347" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="348" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="349" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="350" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="351" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="352" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="353" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="354" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="355" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="356" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="357" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="358" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="359" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="360" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="361" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="362" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="363" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="364" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="365" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="366" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="367" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="368" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="369" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="370" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="371" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="372" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="373" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="374" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="375" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="376" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="377" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="378" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="379" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="380" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="381" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="382" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="383" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="384" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="385" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="386" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="387" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="388" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="389" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="390" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="391" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="392" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="393" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="394" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="395" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="396" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="397" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="398" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="399" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="400" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="401" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="402" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="403" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="404" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="405" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="406" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="407" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="408" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="409" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="410" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="411" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="412" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="413" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="414" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="415" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="416" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="417" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="418" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="419" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="420" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="421" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="422" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="423" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="424" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="425" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="426" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="427" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="428" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="429" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="430" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="431" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="432" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="433" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="434" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="435" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="436" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="437" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="438" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="439" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="440" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="441" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="442" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="443" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="444" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="445" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="446" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="447" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="448" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="449" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="450" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="451" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="452" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="453" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="454" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="455" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="456" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="457" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="458" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="459" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="460" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="461" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="462" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="463" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="464" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="465" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="466" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="467" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="468" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="469" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="470" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="471" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="472" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="473" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="474" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="475" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="476" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="477" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="478" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="479" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="480" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="481" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="482" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="483" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="484" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="485" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="486" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="487" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="488" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="489" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="490" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="491" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="492" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="493" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="494" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="495" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="496" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="497" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="498" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="499" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="500" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="501" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="502" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="503" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="504" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="505" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="506" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="507" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="508" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="509" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="510" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="511" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="512" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="513" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="514" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="515" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="516" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="517" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="518" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="519" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="520" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="521" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="522" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="523" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="524" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="525" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="526" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="527" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="528" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="529" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="530" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="531" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="532" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="533" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="534" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="535" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="536" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="537" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="538" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="539" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="540" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="541" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="542" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="543" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="544" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="545" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="546" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="547" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="548" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="549" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="550" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="551" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="552" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="553" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="554" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="555" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="556" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="557" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="558" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="559" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="560" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="561" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="562" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="563" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="564" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="565" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="566" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="567" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="568" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="569" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="570" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="571" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="572" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="573" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="574" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="575" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="576" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="577" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="578" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="579" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="580" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="581" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="582" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="583" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="584" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="585" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="586" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="587" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="588" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="589" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="590" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="591" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="592" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="593" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="594" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="595" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="596" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="597" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="598" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="599" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="600" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="601" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="602" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="603" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="604" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="605" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="606" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="607" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="608" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="609" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="610" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="611" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="612" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="613" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="614" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="615" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="616" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="617" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="618" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="619" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="620" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="621" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="622" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="623" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="624" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="625" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="626" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="627" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="628" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="629" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="630" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="631" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="632" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="633" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="634" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="635" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="636" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="637" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="638" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="639" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="640" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="641" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="642" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="643" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="644" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="645" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="646" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="647" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="648" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="649" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="650" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="651" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="652" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="653" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="654" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="655" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="656" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="657" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="658" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="659" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="660" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="661" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="662" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="663" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="664" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="665" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="666" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="667" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="668" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="669" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="670" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="671" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="672" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="673" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="674" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="675" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="676" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="677" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="678" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="679" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="680" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="681" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="682" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="683" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="684" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="685" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="686" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="687" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="688" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="689" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="690" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="691" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="692" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="693" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="694" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="695" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="696" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="697" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="698" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="699" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="700" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="701" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="702" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="703" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="704" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="705" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="706" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="707" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="708" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="709" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="710" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="711" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="712" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="713" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="714" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="715" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="716" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="717" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="718" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="719" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="720" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="721" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="722" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="723" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="724" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="725" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="726" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="727" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="728" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="729" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="730" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="731" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="732" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="733" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="734" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="735" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="736" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="737" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="738" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="739" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="740" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="741" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="742" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="743" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="744" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="745" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="746" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="747" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="748" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="749" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="750" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="751" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="752" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="753" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="754" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="755" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="756" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="757" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="758" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="759" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="760" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="761" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="762" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="763" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="764" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="765" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="766" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="767" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="768" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="769" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="770" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="771" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="772" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="773" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="774" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="775" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="776" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="777" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="778" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="779" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="780" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="781" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="782" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="783" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="784" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="785" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="786" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="787" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="788" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="789" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="790" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="791" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="792" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="793" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="794" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="795" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="796" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="797" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="798" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="799" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="800" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="801" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="802" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="803" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="804" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="805" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="806" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="807" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="808" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="809" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="810" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="811" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="812" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="813" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="814" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="815" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="816" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="817" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="818" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="819" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="820" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="821" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="822" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="823" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="824" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="825" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="826" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="827" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="828" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="829" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="830" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="831" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="832" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="833" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="834" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="835" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="836" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="837" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="838" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="839" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="840" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="841" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="842" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="843" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="844" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="845" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="846" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="847" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="848" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="849" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="850" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="851" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="852" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="853" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="854" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="855" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="856" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="857" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="858" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="859" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="860" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="861" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="862" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="863" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="864" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="865" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="866" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="867" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="868" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="869" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="870" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="871" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="872" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="873" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="874" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="875" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="876" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="877" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="878" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="879" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="880" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="881" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="882" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="883" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="884" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="885" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="886" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="887" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="888" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="889" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="890" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="891" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="892" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="893" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="894" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="895" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="896" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="897" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="898" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="899" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="900" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="901" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="902" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="903" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="904" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="905" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="906" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="907" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="908" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="909" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="910" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="911" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="912" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="913" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="914" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="915" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="916" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="917" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="918" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="919" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="920" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="921" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="922" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="923" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="924" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="925" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="926" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="927" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="928" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="929" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="930" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="931" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="932" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="933" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="934" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="935" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="936" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="937" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="938" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="939" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="940" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="941" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="942" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="943" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="944" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="945" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="946" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="947" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="948" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="949" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="950" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="951" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="952" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="953" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="954" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="955" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="956" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="957" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="958" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="959" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="960" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="961" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="962" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="963" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="964" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="965" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="966" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="967" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="968" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="969" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="970" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="971" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="972" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="973" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="974" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="975" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="976" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="977" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="978" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="979" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="980" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="981" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="982" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="983" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="984" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="985" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="986" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="987" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="988" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -3553,6 +3570,27 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6265ed9f-cd81-4be6-845e-c0b4df03a361" xsi:nil="true"/>
+    <EtiquetaSGSI xmlns="e71f9cff-904e-474b-904c-48ca19d2bb89" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e71f9cff-904e-474b-904c-48ca19d2bb89">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101008827B542147F564D9F09914A7F6EA273" ma:contentTypeVersion="17" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="8856ecc99a8eaa98f128264fae8013e0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e71f9cff-904e-474b-904c-48ca19d2bb89" xmlns:ns3="6265ed9f-cd81-4be6-845e-c0b4df03a361" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5efc7a3396158f5d601533948a751157" ns2:_="" ns3:_="">
     <xsd:import namespace="e71f9cff-904e-474b-904c-48ca19d2bb89"/>
@@ -3803,35 +3841,40 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6265ed9f-cd81-4be6-845e-c0b4df03a361" xsi:nil="true"/>
-    <EtiquetaSGSI xmlns="e71f9cff-904e-474b-904c-48ca19d2bb89" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e71f9cff-904e-474b-904c-48ca19d2bb89">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7968044-0414-437A-8CBF-853B86C05442}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3C801364-ADBD-4E1F-BCB7-BA3870F485C3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="6265ed9f-cd81-4be6-845e-c0b4df03a361"/>
+    <ds:schemaRef ds:uri="e71f9cff-904e-474b-904c-48ca19d2bb89"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F6DB233-C399-404D-B8B3-C85C9515927C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F6DB233-C399-404D-B8B3-C85C9515927C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3C801364-ADBD-4E1F-BCB7-BA3870F485C3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7968044-0414-437A-8CBF-853B86C05442}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="e71f9cff-904e-474b-904c-48ca19d2bb89"/>
+    <ds:schemaRef ds:uri="6265ed9f-cd81-4be6-845e-c0b4df03a361"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>